<commit_message>
MTP benchmarks: 48-103% speedup on 4 MTP-capable models
- Gemma-4-E2B: 23.7 → 39.1 tok/s (+65%), separate draft
- Gemma-4-E4B-UD: 15.6 → 31.7 tok/s (+103%), BFCL 92.3% champion now fast
- Qwen3.5-2B: 27.7 → 41.0 tok/s (+48%), embedded MTP at 48K f16
- Qwen3.5-4B: 13.1 → 24.9 tok/s (+90%), embedded MTP
- Added MTP columns to Original Sweep and 32K Retests sheets
- Added MTP discoveries to Discoveries sheet
</commit_message>
<xml_diff>
--- a/32k_retest_results.xlsx
+++ b/32k_retest_results.xlsx
@@ -35,7 +35,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +66,18 @@
         <bgColor rgb="00FCE4EC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EFDF"/>
+        <bgColor rgb="00D4EFDF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADBD8"/>
+        <bgColor rgb="00FADBD8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -85,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -107,6 +119,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -473,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -491,6 +509,8 @@
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -569,6 +589,16 @@
           <t>All Stop?</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>MTP tok/s</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>MTP Speedup</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -626,6 +656,16 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -683,6 +723,16 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -740,6 +790,14 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P4" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>+48%</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -797,6 +855,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -854,6 +922,16 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -911,6 +989,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -968,6 +1056,16 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1025,6 +1123,14 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P9" s="8" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="Q9" s="8" t="inlineStr">
+        <is>
+          <t>+60%</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1082,6 +1188,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1139,6 +1255,16 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1196,6 +1322,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1253,6 +1389,16 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1310,6 +1456,16 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1367,6 +1523,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1424,6 +1590,16 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1481,6 +1657,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1538,6 +1724,16 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1595,6 +1791,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1652,6 +1858,16 @@
       <c r="O20" s="3" t="inlineStr">
         <is>
           <t>❌</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1711,6 +1927,16 @@
           <t>✅</t>
         </is>
       </c>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1768,6 +1994,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1825,6 +2061,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1884,6 +2130,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1943,6 +2199,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -2002,6 +2268,16 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -2059,6 +2335,16 @@
       <c r="O27" s="3" t="inlineStr">
         <is>
           <t>❌</t>
+        </is>
+      </c>
+      <c r="P27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2118,6 +2404,14 @@
           <t>❌</t>
         </is>
       </c>
+      <c r="P28" s="8" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="Q28" s="8" t="inlineStr">
+        <is>
+          <t>+90%</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -2173,6 +2467,16 @@
       <c r="O29" s="3" t="inlineStr">
         <is>
           <t>❌</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:S10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2207,6 +2511,8 @@
     <col width="7" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2295,6 +2601,16 @@
           <t>vs 16K Speed</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>MTP tok/s</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>MTP Speedup</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -2362,6 +2678,14 @@
           <t>97%</t>
         </is>
       </c>
+      <c r="R2" s="8" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="S2" s="8" t="inlineStr">
+        <is>
+          <t>+65%</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -2429,6 +2753,8 @@
           <t>98%</t>
         </is>
       </c>
+      <c r="R3" s="3" t="n"/>
+      <c r="S3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -2496,6 +2822,16 @@
           <t>102%</t>
         </is>
       </c>
+      <c r="R4" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S4" s="9" t="inlineStr">
+        <is>
+          <t>no MTP</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2563,6 +2899,14 @@
       <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>NEW (couldn't load before!)</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>+103%</t>
         </is>
       </c>
     </row>
@@ -2632,6 +2976,16 @@
           <t>91%</t>
         </is>
       </c>
+      <c r="R6" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S6" s="9" t="inlineStr">
+        <is>
+          <t>no MTP</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -2699,6 +3053,16 @@
           <t>—</t>
         </is>
       </c>
+      <c r="R7" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S7" s="9" t="inlineStr">
+        <is>
+          <t>no MTP</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -2768,6 +3132,16 @@
           <t>72%</t>
         </is>
       </c>
+      <c r="R8" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S8" s="9" t="inlineStr">
+        <is>
+          <t>no MTP</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2837,6 +3211,16 @@
           <t>99%</t>
         </is>
       </c>
+      <c r="R9" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S9" s="9" t="inlineStr">
+        <is>
+          <t>no MTP</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2904,6 +3288,16 @@
       <c r="Q10" s="5" t="inlineStr">
         <is>
           <t>65%</t>
+        </is>
+      </c>
+      <c r="R10" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S10" s="9" t="inlineStr">
+        <is>
+          <t>no MTP</t>
         </is>
       </c>
     </row>
@@ -21370,7 +21764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -21548,6 +21942,108 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>MTP Multi-Token Prediction</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Game-changer</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>MTP speculative decoding gives 48-103% speedup with zero quality loss. 4 of our models support it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Gemma-4-E2B + MTP</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Best speed</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>23.7 → 39.1 tok/s (+65%). Separate draft model (93MB). All 12 tests stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Gemma-4-E4B-UD + MTP</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Best tool model</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>15.6 → 31.7 tok/s (+103%!). BFCL 92.3% champion now FAST. Separate draft (57MB).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Qwen3.5-2B + MTP</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Fastest overall</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>27.7 → 41.0 tok/s (+48%). Embedded MTP (no draft needed). 48K f16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Qwen3.5-4B + MTP</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Biggest gain</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>13.1 → 24.9 tok/s (+90%). Embedded MTP. 2 func errors under memory pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>MTP types</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Embedded (Qwen3.5): nextn_predict_layers in GGUF, --spec-type draft-mtp alone. Separate (Gemma-4): needs --model-draft companion file.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Spark 32K q8_0: 14.4 t/s, same speed as 16K, no -nkvo needed
q8_0 KV pre-allocates larger but avoids the memory fragmentation that
killed q4_0 at 32K. Best Spark config: 2× context, better KV quality,
zero speed penalty.
</commit_message>
<xml_diff>
--- a/32k_retest_results.xlsx
+++ b/32k_retest_results.xlsx
@@ -35,7 +35,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -78,6 +78,12 @@
         <bgColor rgb="00FADBD8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -97,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -124,6 +130,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2491,7 +2500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3296,6 +3305,85 @@
         </is>
       </c>
       <c r="S10" s="9" t="inlineStr">
+        <is>
+          <t>no MTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>spark-x2.5-4b-32k-q8</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Q4_K_M</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>spark2_5</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>90.40000000000001</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>32768</v>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>q8_0</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>NO_PINNED only</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="10" t="inlineStr">
+        <is>
+          <t>⚠️</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>99% of 16K</t>
+        </is>
+      </c>
+      <c r="R11" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S11" s="10" t="inlineStr">
         <is>
           <t>no MTP</t>
         </is>
@@ -21764,7 +21852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -22044,6 +22132,23 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Spark 32K q8_0 breakthrough</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Best Spark config</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Spark-X2.5-4B at 32K with q8_0 KV runs at 14.4 t/s (same as 16K!) with NO -nkvo needed. q8_0 KV pre-allocates more upfront but avoids the fragmentation that killed q4_0 at 32K. Better quality than q4_0 + full speed + 2× context.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BFCL + poetry benchmarks for 6 models with new settings
Results sheet 'BFCL + Poetry' added to spreadsheet:
- Spark-X2.5-4B: 47/52 (90.4%), 14.4 t/s, full run survived
- Gemma-4-E2B: 45/52 (86.5%), 24.3 t/s, full run survived
- Gemma-4-E4B-UD: 48/52 (92.3%), 15.2 t/s, died on coding
- Qwen3.5-2B: 45/52 (86.5%), 27.5 t/s, 12/12 parallel, died on coding
- Qwen3.5-4B: 13/52 (25.0%), 13.4 t/s, crashed early
- Hermes-3-3B: 1/52 (1.9%), 18.0 t/s, stable but no tool calling

Key finding: only Spark and Gemma-4-E2B survive full 52-test BFCL at 32K.
Coding tests (4096-token gens) kill servers under multi-turn memory pressure.
</commit_message>
<xml_diff>
--- a/32k_retest_results.xlsx
+++ b/32k_retest_results.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Per-Test Detail" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Architecture &amp; KV" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Discoveries" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="BFCL + Poetry" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35,7 +36,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +85,18 @@
         <bgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCDD2"/>
+        <bgColor rgb="00FFCDD2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -103,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -134,6 +147,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -22152,4 +22183,478 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>BFCL Score</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>BFCL %</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Parallel</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Chained</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Coding</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Server survived?</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Poetry tok/s</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Poetry tokens</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Poetry finish</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Best use case</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Spark-X2.5-4B</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>32K q8_0</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>47/52</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>90.4%</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>28/30</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>7/8</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Yes - full run</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="K2" s="11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L2" s="11" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="M2" s="12" t="inlineStr">
+        <is>
+          <t>Best tool model at 32K - stable, high accuracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Gemma-4-E2B</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>32K q4_0</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>45/52</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>86.5%</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>28/30</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>5/8</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Yes - full run</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="K3" s="11" t="n">
+        <v>769</v>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="M3" s="12" t="inlineStr">
+        <is>
+          <t>Fast + stable all-rounder (39.1 t/s with MTP!)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Gemma-4-E4B-UD</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>16K q8_0</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>48/52</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>92.3%</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>28/30</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>11/12</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>Died on 2nd coding test</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="K4" s="13" t="n">
+        <v>531</v>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="inlineStr">
+        <is>
+          <t>BFCL champion - best accuracy (31.7 t/s with MTP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Qwen3.5-2B</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>48K f16</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>45/52</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>86.5%</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>26/30</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>7/8</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>Died on coding tests</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="M5" s="14" t="inlineStr">
+        <is>
+          <t>100% parallel! Fastest (41.0 t/s with MTP). 48K ctx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Qwen3.5-4B</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>16K q4_0</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>13/52</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>25.0%</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>13/30</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>0/12</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>0/8</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="inlineStr">
+        <is>
+          <t>Crashed after 13 tests</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="K6" s="15" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="M6" s="16" t="inlineStr">
+        <is>
+          <t>MTP speed (24.9 t/s) but not viable for multi-turn BFCL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Hermes-3-3B</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>32K q4_0</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>1/52</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>1.9%</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>0/30</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>0/12</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>0/8</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="I7" s="15" t="inlineStr">
+        <is>
+          <t>Yes - full run (stable)</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="K7" s="15" t="n">
+        <v>78</v>
+      </c>
+      <c r="L7" s="15" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>Stable but no tool calling. Good for chat/poetry only</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Coding retests: E4B-UD needs 32K q4_0 (not 16K q8_0) for full BFCL
Fix: E4B-UD crashed on 2nd coding test at 16K q8_0 (KV too small for
sequential 6K-char generations). At 32K q4_0 both coding tests pass
(3/4 python, 6/7 html = 2/2). Updated launch script to use q4_0 KV.

Qwen3.5-2B (48K f16) and Qwen3.5-4B (16K q4_0) both survived coding
tests with capped max_tokens (16000/12000). Remaining failures are
quality, not crashes.

Root cause: default max_tokens=16384 overflows 16K context window.
Capping at 12000 for 16K models, 16000 for 48K models fixes crashes.
</commit_message>
<xml_diff>
--- a/32k_retest_results.xlsx
+++ b/32k_retest_results.xlsx
@@ -116,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -165,6 +165,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3342,79 +3345,79 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>spark-x2.5-4b-32k-q8</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>4B</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Q4_K_M</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>spark2_5</t>
         </is>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="11" t="n">
         <v>2600</v>
       </c>
-      <c r="F11" s="10" t="n">
+      <c r="F11" s="11" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="G11" s="10" t="n">
+      <c r="G11" s="11" t="n">
         <v>32768</v>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>q8_0</t>
         </is>
       </c>
-      <c r="I11" s="10" t="inlineStr">
+      <c r="I11" s="11" t="inlineStr">
         <is>
           <t>NO_PINNED only</t>
         </is>
       </c>
-      <c r="J11" s="10" t="n">
+      <c r="J11" s="11" t="n">
         <v>14.4</v>
       </c>
-      <c r="K11" s="10" t="n">
+      <c r="K11" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="L11" s="10" t="n">
+      <c r="L11" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="M11" s="10" t="n">
+      <c r="M11" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="N11" s="10" t="n">
+      <c r="N11" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="O11" s="10" t="n">
+      <c r="O11" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="P11" s="10" t="inlineStr">
+      <c r="P11" s="11" t="inlineStr">
         <is>
           <t>⚠️</t>
         </is>
       </c>
-      <c r="Q11" s="10" t="inlineStr">
+      <c r="Q11" s="11" t="inlineStr">
         <is>
           <t>99% of 16K</t>
         </is>
       </c>
-      <c r="R11" s="10" t="inlineStr">
+      <c r="R11" s="11" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="S11" s="10" t="inlineStr">
+      <c r="S11" s="11" t="inlineStr">
         <is>
           <t>no MTP</t>
         </is>
@@ -22191,7 +22194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -22202,9 +22205,9 @@
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="42" customWidth="1" min="13" max="13"/>
   </cols>
@@ -22252,25 +22255,40 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Coding (retest)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Coding max_tokens</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Retest config</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Server survived?</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Poetry tok/s</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Poetry tokens</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Poetry finish</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Best use case</t>
         </is>
@@ -22317,23 +22335,38 @@
           <t>2/2</t>
         </is>
       </c>
-      <c r="I2" s="11" t="inlineStr">
+      <c r="I2" s="17" t="inlineStr">
+        <is>
+          <t>2/2 (100%)</t>
+        </is>
+      </c>
+      <c r="J2" s="17" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="K2" s="17" t="inlineStr">
+        <is>
+          <t>32K q8_0 — already worked</t>
+        </is>
+      </c>
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>Yes - full run</t>
         </is>
       </c>
-      <c r="J2" s="11" t="n">
+      <c r="M2" s="11" t="n">
         <v>14.4</v>
       </c>
-      <c r="K2" s="11" t="n">
-        <v>1024</v>
-      </c>
-      <c r="L2" s="11" t="inlineStr">
+      <c r="N2" s="11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="O2" s="11" t="inlineStr">
         <is>
           <t>length</t>
         </is>
       </c>
-      <c r="M2" s="12" t="inlineStr">
+      <c r="P2" s="12" t="inlineStr">
         <is>
           <t>Best tool model at 32K - stable, high accuracy</t>
         </is>
@@ -22380,23 +22413,38 @@
           <t>2/2</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>2/2 (100%)</t>
+        </is>
+      </c>
+      <c r="J3" s="17" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="K3" s="17" t="inlineStr">
+        <is>
+          <t>32K q4_0 — already worked</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
         <is>
           <t>Yes - full run</t>
         </is>
       </c>
-      <c r="J3" s="11" t="n">
+      <c r="M3" s="11" t="n">
         <v>24.3</v>
       </c>
-      <c r="K3" s="11" t="n">
+      <c r="N3" s="11" t="n">
         <v>769</v>
       </c>
-      <c r="L3" s="11" t="inlineStr">
-        <is>
-          <t>stop</t>
-        </is>
-      </c>
-      <c r="M3" s="12" t="inlineStr">
+      <c r="O3" s="11" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="P3" s="12" t="inlineStr">
         <is>
           <t>Fast + stable all-rounder (39.1 t/s with MTP!)</t>
         </is>
@@ -22443,25 +22491,38 @@
           <t>1/2</t>
         </is>
       </c>
-      <c r="I4" s="13" t="inlineStr">
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>2/2 (100%)</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="n">
+        <v>12000</v>
+      </c>
+      <c r="K4" s="17" t="inlineStr">
+        <is>
+          <t>32K q4_0 (was 16K q8_0)</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
         <is>
           <t>Died on 2nd coding test</t>
         </is>
       </c>
-      <c r="J4" s="13" t="n">
+      <c r="M4" s="13" t="n">
         <v>15.2</v>
       </c>
-      <c r="K4" s="13" t="n">
+      <c r="N4" s="13" t="n">
         <v>531</v>
       </c>
-      <c r="L4" s="13" t="inlineStr">
-        <is>
-          <t>stop</t>
-        </is>
-      </c>
-      <c r="M4" s="14" t="inlineStr">
-        <is>
-          <t>BFCL champion - best accuracy (31.7 t/s with MTP)</t>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="P4" s="14" t="inlineStr">
+        <is>
+          <t>BFCL champion 92.3% — use 32K q4_0 for full BFCL (coding 2/2)</t>
         </is>
       </c>
     </row>
@@ -22506,23 +22567,36 @@
           <t>0/2</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>1/2 (50%)</t>
+        </is>
+      </c>
+      <c r="J5" s="17" t="n">
+        <v>16000</v>
+      </c>
+      <c r="K5" s="17" t="inlineStr">
+        <is>
+          <t>48K f16 — survived, quality issue</t>
+        </is>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
         <is>
           <t>Died on coding tests</t>
         </is>
       </c>
-      <c r="J5" s="13" t="n">
+      <c r="M5" s="13" t="n">
         <v>27.5</v>
       </c>
-      <c r="K5" s="13" t="n">
-        <v>1024</v>
-      </c>
-      <c r="L5" s="13" t="inlineStr">
+      <c r="N5" s="13" t="n">
+        <v>1024</v>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
         <is>
           <t>length</t>
         </is>
       </c>
-      <c r="M5" s="14" t="inlineStr">
+      <c r="P5" s="14" t="inlineStr">
         <is>
           <t>100% parallel! Fastest (41.0 t/s with MTP). 48K ctx</t>
         </is>
@@ -22569,23 +22643,36 @@
           <t>0/2</t>
         </is>
       </c>
-      <c r="I6" s="15" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>1/2 (50%)</t>
+        </is>
+      </c>
+      <c r="J6" s="17" t="n">
+        <v>12000</v>
+      </c>
+      <c r="K6" s="17" t="inlineStr">
+        <is>
+          <t>16K q4_0 — survived, quality issue</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
         <is>
           <t>Crashed after 13 tests</t>
         </is>
       </c>
-      <c r="J6" s="15" t="n">
+      <c r="M6" s="15" t="n">
         <v>13.4</v>
       </c>
-      <c r="K6" s="15" t="n">
-        <v>1024</v>
-      </c>
-      <c r="L6" s="15" t="inlineStr">
+      <c r="N6" s="15" t="n">
+        <v>1024</v>
+      </c>
+      <c r="O6" s="15" t="inlineStr">
         <is>
           <t>length</t>
         </is>
       </c>
-      <c r="M6" s="16" t="inlineStr">
+      <c r="P6" s="16" t="inlineStr">
         <is>
           <t>MTP speed (24.9 t/s) but not viable for multi-turn BFCL</t>
         </is>
@@ -22632,23 +22719,38 @@
           <t>1/2</t>
         </is>
       </c>
-      <c r="I7" s="15" t="inlineStr">
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>1/2 (50%)</t>
+        </is>
+      </c>
+      <c r="J7" s="17" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="K7" s="17" t="inlineStr">
+        <is>
+          <t>32K q4_0 — already worked, quality issue</t>
+        </is>
+      </c>
+      <c r="L7" s="15" t="inlineStr">
         <is>
           <t>Yes - full run (stable)</t>
         </is>
       </c>
-      <c r="J7" s="15" t="n">
+      <c r="M7" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="K7" s="15" t="n">
+      <c r="N7" s="15" t="n">
         <v>78</v>
       </c>
-      <c r="L7" s="15" t="inlineStr">
-        <is>
-          <t>stop</t>
-        </is>
-      </c>
-      <c r="M7" s="16" t="inlineStr">
+      <c r="O7" s="15" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="P7" s="16" t="inlineStr">
         <is>
           <t>Stable but no tool calling. Good for chat/poetry only</t>
         </is>

</xml_diff>